<commit_message>
fix: remove unused CSV file generation code
</commit_message>
<xml_diff>
--- a/Code Real/data/3_Data_Normalized/Hasil_ZScore_Data_Normalization.xlsx
+++ b/Code Real/data/3_Data_Normalized/Hasil_ZScore_Data_Normalization.xlsx
@@ -487,19 +487,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.1929512760917949</v>
+        <v>-0.1929512760917947</v>
       </c>
       <c r="C2" t="n">
-        <v>0.451346025238293</v>
+        <v>0.4513460252382928</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0510525786323969</v>
+        <v>0.05105257863239707</v>
       </c>
       <c r="E2" t="n">
         <v>-0.3272078578808691</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.4749628217465232</v>
+        <v>-0.4749628217465233</v>
       </c>
       <c r="G2" t="n">
         <v>-0.07669649888473706</v>
@@ -508,7 +508,7 @@
         <v>-0.1891480179719353</v>
       </c>
       <c r="I2" t="n">
-        <v>0.05495021041385634</v>
+        <v>0.05495021041385652</v>
       </c>
       <c r="J2" t="n">
         <v>-0.2883807434472616</v>
@@ -521,13 +521,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.3939834389979133</v>
+        <v>-0.393983438997913</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8456701852990859</v>
+        <v>0.8456701852990861</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.7903504530819332</v>
+        <v>-0.7903504530819327</v>
       </c>
       <c r="E3" t="n">
         <v>-0.5997575131036713</v>
@@ -545,7 +545,7 @@
         <v>0.4185247954472307</v>
       </c>
       <c r="J3" t="n">
-        <v>-0.2412343942988228</v>
+        <v>-0.2412343942988227</v>
       </c>
     </row>
     <row r="4">
@@ -555,13 +555,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.4362496462204831</v>
+        <v>-0.4362496462204829</v>
       </c>
       <c r="C4" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.7449806817640036</v>
+        <v>-0.7449806817640034</v>
       </c>
       <c r="E4" t="n">
         <v>-0.02831173598652924</v>
@@ -589,13 +589,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.4229538058055874</v>
+        <v>-0.4229538058055875</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1820147369918203</v>
+        <v>0.1820147369918201</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.6625743624314376</v>
+        <v>-0.6625743624314374</v>
       </c>
       <c r="E5" t="n">
         <v>0.079799627251849</v>
@@ -629,7 +629,7 @@
         <v>1.461924971914749</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.1616550505334808</v>
+        <v>-0.1616550505334806</v>
       </c>
       <c r="E6" t="n">
         <v>-0.07155628128188057</v>
@@ -657,13 +657,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.1348412313950073</v>
+        <v>-0.1348412313950074</v>
       </c>
       <c r="C7" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.5181318251743557</v>
+        <v>-0.5181318251743556</v>
       </c>
       <c r="E7" t="n">
         <v>-0.1462514049738509</v>
@@ -691,13 +691,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-0.2219710588739683</v>
+        <v>-0.2219710588739684</v>
       </c>
       <c r="C8" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.6418675651323453</v>
+        <v>-0.6418675651323452</v>
       </c>
       <c r="E8" t="n">
         <v>0.06628570684705171</v>
@@ -731,7 +731,7 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.6847962912402195</v>
+        <v>-0.6847962912402192</v>
       </c>
       <c r="E9" t="n">
         <v>-0.4247200678605828</v>
@@ -759,13 +759,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.3501174954642522</v>
+        <v>-0.3501174954642519</v>
       </c>
       <c r="C10" t="n">
         <v>0.3250656607784866</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.4403550743436194</v>
+        <v>-0.4403550743436192</v>
       </c>
       <c r="E10" t="n">
         <v>-0.05920069691178016</v>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-0.3442124338362751</v>
+        <v>-0.3442124338362753</v>
       </c>
       <c r="C11" t="n">
         <v>1.153308575779632</v>
@@ -827,16 +827,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.375368890629648</v>
+        <v>-0.3753688906296477</v>
       </c>
       <c r="C12" t="n">
         <v>0.07470869078285895</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.4834100614106342</v>
+        <v>-0.4834100614106341</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.4017873544463813</v>
+        <v>-0.4017873544463814</v>
       </c>
       <c r="F12" t="n">
         <v>-1.000382558752324</v>
@@ -861,13 +861,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.3262116535064206</v>
+        <v>-0.3262116535064205</v>
       </c>
       <c r="C13" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.6602239661151241</v>
+        <v>-0.660223966115124</v>
       </c>
       <c r="E13" t="n">
         <v>-0.4762016694026677</v>
@@ -901,13 +901,13 @@
         <v>0.8029724331479404</v>
       </c>
       <c r="D14" t="n">
-        <v>2.527462882100652</v>
+        <v>2.527462882100653</v>
       </c>
       <c r="E14" t="n">
         <v>0.1380134382263603</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.5881301497170034</v>
+        <v>-0.5881301497170033</v>
       </c>
       <c r="G14" t="n">
         <v>-0.07669649888473706</v>
@@ -935,10 +935,10 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.487430476162223</v>
+        <v>-0.4874304761622229</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.3346272651619343</v>
+        <v>-0.3346272651619342</v>
       </c>
       <c r="F15" t="n">
         <v>-1.000382558752324</v>
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.3535966902941718</v>
+        <v>-0.3535966902941717</v>
       </c>
       <c r="C16" t="n">
         <v>-0.116191757780307</v>
@@ -1003,7 +1003,7 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D17" t="n">
-        <v>-1.101457456404879</v>
+        <v>-1.101457456404878</v>
       </c>
       <c r="E17" t="n">
         <v>-0.6445465064452852</v>
@@ -1031,13 +1031,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-0.3556067701659631</v>
+        <v>-0.355606770165963</v>
       </c>
       <c r="C18" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D18" t="n">
-        <v>0.06519380605616706</v>
+        <v>0.06519380605616724</v>
       </c>
       <c r="E18" t="n">
         <v>-0.4367324415537359</v>
@@ -1065,13 +1065,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-0.1459342287445163</v>
+        <v>-0.1459342287445164</v>
       </c>
       <c r="C19" t="n">
-        <v>0.06998890547318484</v>
+        <v>0.06998890547318509</v>
       </c>
       <c r="D19" t="n">
-        <v>0.474910618468082</v>
+        <v>0.4749106184680822</v>
       </c>
       <c r="E19" t="n">
         <v>1.139290986987956</v>
@@ -1099,13 +1099,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.4507522602659166</v>
+        <v>0.4507522602659165</v>
       </c>
       <c r="C20" t="n">
-        <v>0.2755576270462177</v>
+        <v>0.2755576270462178</v>
       </c>
       <c r="D20" t="n">
-        <v>0.8547456705500061</v>
+        <v>0.8547456705500062</v>
       </c>
       <c r="E20" t="n">
         <v>2.296082573638603</v>
@@ -1133,13 +1133,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.4297847183650136</v>
+        <v>0.429784718365014</v>
       </c>
       <c r="C21" t="n">
         <v>0.07470869078285895</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.3187042589416984</v>
+        <v>-0.3187042589416981</v>
       </c>
       <c r="E21" t="n">
         <v>1.009557351101902</v>
@@ -1167,16 +1167,16 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-0.3869599362647534</v>
+        <v>-0.3869599362647535</v>
       </c>
       <c r="C22" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.3917446050744092</v>
+        <v>-0.391744605074409</v>
       </c>
       <c r="E22" t="n">
-        <v>-0.5106547412039091</v>
+        <v>-0.510654741203909</v>
       </c>
       <c r="F22" t="n">
         <v>-0.1758777406816829</v>
@@ -1201,13 +1201,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-0.4037193698196007</v>
+        <v>-0.4037193698196006</v>
       </c>
       <c r="C23" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.7125737022511967</v>
+        <v>-0.7125737022511965</v>
       </c>
       <c r="E23" t="n">
         <v>-0.6409427943373392</v>
@@ -1238,16 +1238,16 @@
         <v>-0.4086481430313368</v>
       </c>
       <c r="C24" t="n">
-        <v>0.9900086017312377</v>
+        <v>0.9900086017312379</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.8195167346434592</v>
+        <v>-0.819516734643459</v>
       </c>
       <c r="E24" t="n">
         <v>-0.5497900763128243</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.2122529532436229</v>
+        <v>-0.2122529532436228</v>
       </c>
       <c r="G24" t="n">
         <v>-0.07669649888473706</v>
@@ -1269,19 +1269,19 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>-0.4198809013368314</v>
+        <v>-0.4198809013368311</v>
       </c>
       <c r="C25" t="n">
-        <v>0.9900086017312377</v>
+        <v>0.9900086017312379</v>
       </c>
       <c r="D25" t="n">
-        <v>0.3535041755149311</v>
+        <v>0.3535041755149314</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.4925546487160358</v>
+        <v>-0.4925546487160359</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.5275047954471033</v>
+        <v>-0.5275047954471034</v>
       </c>
       <c r="G25" t="n">
         <v>-0.07669649888473706</v>
@@ -1303,19 +1303,19 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>-0.3703366805734313</v>
+        <v>-0.3703366805734311</v>
       </c>
       <c r="C26" t="n">
-        <v>1.076633599445614</v>
+        <v>1.076633599445615</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.3198773622724787</v>
+        <v>-0.3198773622724785</v>
       </c>
       <c r="E26" t="n">
         <v>-0.0965925969791892</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.7183151209913151</v>
+        <v>-0.7183151209913153</v>
       </c>
       <c r="G26" t="n">
         <v>-0.07669649888473706</v>
@@ -1340,16 +1340,16 @@
         <v>-0.3557894944837095</v>
       </c>
       <c r="C27" t="n">
-        <v>-0.05035268422886165</v>
+        <v>-0.05035268422886203</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.01557435826805923</v>
+        <v>-0.01557435826805905</v>
       </c>
       <c r="E27" t="n">
         <v>-0.007719095369695271</v>
       </c>
       <c r="F27" t="n">
-        <v>-0.6175767503623835</v>
+        <v>-0.6175767503623837</v>
       </c>
       <c r="G27" t="n">
         <v>-0.07669649888473706</v>
@@ -1371,13 +1371,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>-0.3685090373541951</v>
+        <v>-0.3685090373541949</v>
       </c>
       <c r="C28" t="n">
-        <v>0.1820147369918203</v>
+        <v>0.1820147369918201</v>
       </c>
       <c r="D28" t="n">
-        <v>-0.1813665122990024</v>
+        <v>-0.1813665122990022</v>
       </c>
       <c r="E28" t="n">
         <v>-0.06010919576252283</v>
@@ -1411,13 +1411,13 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.7287771920076</v>
+        <v>-0.7287771920075998</v>
       </c>
       <c r="E29" t="n">
         <v>-0.267294749460839</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.7183151209913151</v>
+        <v>-0.7183151209913153</v>
       </c>
       <c r="G29" t="n">
         <v>-0.07669649888473706</v>
@@ -1439,16 +1439,16 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>-0.4227746672381499</v>
+        <v>-0.4227746672381497</v>
       </c>
       <c r="C30" t="n">
-        <v>0.4179729220835761</v>
+        <v>0.4179729220835757</v>
       </c>
       <c r="D30" t="n">
         <v>0.2366474809170268</v>
       </c>
       <c r="E30" t="n">
-        <v>0.6139969514885415</v>
+        <v>0.6139969514885421</v>
       </c>
       <c r="F30" t="n">
         <v>-1.000382558752324</v>
@@ -1473,7 +1473,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>-0.4155735797878373</v>
+        <v>-0.4155735797878372</v>
       </c>
       <c r="C31" t="n">
         <v>-0.625979127747597</v>
@@ -1507,19 +1507,19 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>-0.3359600166954212</v>
+        <v>-0.3359600166954211</v>
       </c>
       <c r="C32" t="n">
-        <v>0.9900086017312377</v>
+        <v>0.9900086017312379</v>
       </c>
       <c r="D32" t="n">
-        <v>0.3879272308950474</v>
+        <v>0.3879272308950477</v>
       </c>
       <c r="E32" t="n">
         <v>-0.06010919576252283</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.5275047954471033</v>
+        <v>-0.5275047954471034</v>
       </c>
       <c r="G32" t="n">
         <v>-0.07669649888473706</v>
@@ -1541,13 +1541,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>-0.380463882577161</v>
+        <v>-0.3804638825771607</v>
       </c>
       <c r="C33" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.4124568919804204</v>
+        <v>-0.4124568919804203</v>
       </c>
       <c r="E33" t="n">
         <v>-0.0553395767961238</v>
@@ -1575,10 +1575,10 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>-0.03150120345484424</v>
+        <v>-0.03150120345484436</v>
       </c>
       <c r="C34" t="n">
-        <v>0.1820147369918203</v>
+        <v>0.1820147369918201</v>
       </c>
       <c r="D34" t="n">
         <v>3.503279723460309</v>
@@ -1609,13 +1609,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>-0.08823690506905144</v>
+        <v>-0.0882369050690515</v>
       </c>
       <c r="C35" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.7644248694716876</v>
+        <v>-0.7644248694716875</v>
       </c>
       <c r="E35" t="n">
         <v>0.944690533158875</v>
@@ -1643,13 +1643,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>-0.1459342287445163</v>
+        <v>-0.1459342287445164</v>
       </c>
       <c r="C36" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.1126998261630704</v>
+        <v>-0.1126998261630703</v>
       </c>
       <c r="E36" t="n">
         <v>1.355513713464712</v>
@@ -1677,13 +1677,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>-0.05342181544215181</v>
+        <v>-0.05342181544215145</v>
       </c>
       <c r="C37" t="n">
-        <v>0.5418339031364962</v>
+        <v>0.5418339031364959</v>
       </c>
       <c r="D37" t="n">
-        <v>-0.194659393723943</v>
+        <v>-0.1946593937239428</v>
       </c>
       <c r="E37" t="n">
         <v>2.674472344972927</v>
@@ -1711,7 +1711,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.08906216247534604</v>
+        <v>0.08906216247534592</v>
       </c>
       <c r="C38" t="n">
         <v>-0.625979127747597</v>
@@ -1782,16 +1782,16 @@
         <v>-0.3872828978819488</v>
       </c>
       <c r="C40" t="n">
-        <v>0.5266769062462705</v>
+        <v>0.5266769062462703</v>
       </c>
       <c r="D40" t="n">
-        <v>-0.0944875119901772</v>
+        <v>-0.09448751199017703</v>
       </c>
       <c r="E40" t="n">
         <v>0.2026534491136425</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.634977014380108</v>
+        <v>-0.6349770143801081</v>
       </c>
       <c r="G40" t="n">
         <v>-0.07669649888473706</v>
@@ -1813,13 +1813,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>-0.3589657522866308</v>
+        <v>-0.3589657522866306</v>
       </c>
       <c r="C41" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D41" t="n">
-        <v>0.0194427761557339</v>
+        <v>0.01944277615573407</v>
       </c>
       <c r="E41" t="n">
         <v>-0.3094012804063127</v>
@@ -1847,10 +1847,10 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>-0.3322219945202617</v>
+        <v>-0.3322219945202618</v>
       </c>
       <c r="C42" t="n">
-        <v>0.4179729220835761</v>
+        <v>0.4179729220835757</v>
       </c>
       <c r="D42" t="n">
         <v>1.103093014777143</v>
@@ -1868,7 +1868,7 @@
         <v>-0.1891480179719353</v>
       </c>
       <c r="I42" t="n">
-        <v>5.71402908116713</v>
+        <v>5.714029081167132</v>
       </c>
       <c r="J42" t="n">
         <v>-0.2883807434472616</v>
@@ -1884,10 +1884,10 @@
         <v>-0.3851537435167356</v>
       </c>
       <c r="C43" t="n">
-        <v>0.393595612186983</v>
+        <v>0.3935956121869834</v>
       </c>
       <c r="D43" t="n">
-        <v>0.02084741303864189</v>
+        <v>0.02084741303864206</v>
       </c>
       <c r="E43" t="n">
         <v>0.09331354765664628</v>
@@ -1915,13 +1915,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>-0.3913364802311043</v>
+        <v>-0.3913364802311044</v>
       </c>
       <c r="C44" t="n">
         <v>-0.277995111137206</v>
       </c>
       <c r="D44" t="n">
-        <v>-0.4583035553045586</v>
+        <v>-0.4583035553045585</v>
       </c>
       <c r="E44" t="n">
         <v>-0.03814004173547271</v>
@@ -1936,7 +1936,7 @@
         <v>-0.1891480179719353</v>
       </c>
       <c r="I44" t="n">
-        <v>3.765077814213699</v>
+        <v>3.7650778142137</v>
       </c>
       <c r="J44" t="n">
         <v>-0.2883807434472616</v>
@@ -1949,10 +1949,10 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>-0.3496890558066867</v>
+        <v>-0.3496890558066866</v>
       </c>
       <c r="C45" t="n">
-        <v>0.4179729220835761</v>
+        <v>0.4179729220835757</v>
       </c>
       <c r="D45" t="n">
         <v>1.496286021341716</v>
@@ -1983,13 +1983,13 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.3999887377689941</v>
+        <v>0.3999887377689945</v>
       </c>
       <c r="C46" t="n">
-        <v>-0.05535225463194691</v>
+        <v>-0.05535225463194678</v>
       </c>
       <c r="D46" t="n">
-        <v>0.6923126528445366</v>
+        <v>0.6923126528445371</v>
       </c>
       <c r="E46" t="n">
         <v>0.8230652495156994</v>
@@ -2017,13 +2017,13 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>-0.1637319918944081</v>
+        <v>-0.1637319918944078</v>
       </c>
       <c r="C47" t="n">
         <v>-0.313404432944867</v>
       </c>
       <c r="D47" t="n">
-        <v>0.3726221792722533</v>
+        <v>0.3726221792722536</v>
       </c>
       <c r="E47" t="n">
         <v>0.9230682605111994</v>
@@ -2035,7 +2035,7 @@
         <v>-0.07669649888473706</v>
       </c>
       <c r="H47" t="n">
-        <v>4.952597852682229</v>
+        <v>4.95259785268223</v>
       </c>
       <c r="I47" t="n">
         <v>-0.2709393764064</v>
@@ -2051,13 +2051,13 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>-0.3656222039166683</v>
+        <v>-0.3656222039166684</v>
       </c>
       <c r="C48" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D48" t="n">
-        <v>-0.1174637148341987</v>
+        <v>-0.1174637148341983</v>
       </c>
       <c r="E48" t="n">
         <v>-0.4985961660734746</v>
@@ -2072,7 +2072,7 @@
         <v>0.8988664666033487</v>
       </c>
       <c r="I48" t="n">
-        <v>2.415147149774212</v>
+        <v>2.415147149774213</v>
       </c>
       <c r="J48" t="n">
         <v>-0.2883807434472616</v>
@@ -2085,13 +2085,13 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>-0.3540787711610391</v>
+        <v>-0.3540787711610389</v>
       </c>
       <c r="C49" t="n">
         <v>-0.1395183485495367</v>
       </c>
       <c r="D49" t="n">
-        <v>0.235663396918055</v>
+        <v>0.2356633969180552</v>
       </c>
       <c r="E49" t="n">
         <v>0.04048640425607512</v>
@@ -2125,7 +2125,7 @@
         <v>9.092892212194817</v>
       </c>
       <c r="D50" t="n">
-        <v>-0.3371928562278511</v>
+        <v>-0.3371928562278509</v>
       </c>
       <c r="E50" t="n">
         <v>-0.2445344624632857</v>
@@ -2153,13 +2153,13 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1.489452028279863</v>
+        <v>1.489452028279864</v>
       </c>
       <c r="C51" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D51" t="n">
-        <v>-0.6698913389904267</v>
+        <v>-0.6698913389904266</v>
       </c>
       <c r="E51" t="n">
         <v>0.06178106671211925</v>
@@ -2187,13 +2187,13 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>-0.365368986030756</v>
+        <v>-0.3653689860307557</v>
       </c>
       <c r="C52" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D52" t="n">
-        <v>-0.7320178899588808</v>
+        <v>-0.7320178899588806</v>
       </c>
       <c r="E52" t="n">
         <v>-0.4967943100195016</v>
@@ -2221,13 +2221,13 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>-0.3911478543652425</v>
+        <v>-0.3911478543652423</v>
       </c>
       <c r="C53" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D53" t="n">
-        <v>-0.5004552908946429</v>
+        <v>-0.5004552908946428</v>
       </c>
       <c r="E53" t="n">
         <v>-0.4391349162923665</v>
@@ -2255,19 +2255,19 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>-0.3682703820307945</v>
+        <v>-0.3682703820307947</v>
       </c>
       <c r="C54" t="n">
         <v>0.8235219456404457</v>
       </c>
       <c r="D54" t="n">
-        <v>0.5135427944615042</v>
+        <v>0.5135427944615044</v>
       </c>
       <c r="E54" t="n">
-        <v>0.5602945749779745</v>
+        <v>0.560294574977974</v>
       </c>
       <c r="F54" t="n">
-        <v>-0.5537757822973934</v>
+        <v>-0.5537757822973935</v>
       </c>
       <c r="G54" t="n">
         <v>-0.07669649888473706</v>
@@ -2289,13 +2289,13 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>-0.3858642458573923</v>
+        <v>-0.3858642458573924</v>
       </c>
       <c r="C55" t="n">
-        <v>0.5860116693615292</v>
+        <v>0.5860116693615289</v>
       </c>
       <c r="D55" t="n">
-        <v>0.3559962593834778</v>
+        <v>0.355996259383478</v>
       </c>
       <c r="E55" t="n">
         <v>0.08655658745424763</v>
@@ -2323,19 +2323,19 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>-0.3781208805041411</v>
+        <v>-0.3781208805041412</v>
       </c>
       <c r="C56" t="n">
-        <v>0.9900086017312377</v>
+        <v>0.9900086017312379</v>
       </c>
       <c r="D56" t="n">
-        <v>0.9796481784472511</v>
+        <v>0.9796481784472502</v>
       </c>
       <c r="E56" t="n">
         <v>0.05096993038828147</v>
       </c>
       <c r="F56" t="n">
-        <v>-0.285811716424435</v>
+        <v>-0.2858117164244349</v>
       </c>
       <c r="G56" t="n">
         <v>-0.07669649888473706</v>
@@ -2363,13 +2363,13 @@
         <v>1.120827038618624</v>
       </c>
       <c r="D57" t="n">
-        <v>-0.369440977997948</v>
+        <v>-0.3694409779979478</v>
       </c>
       <c r="E57" t="n">
         <v>-0.151867579687533</v>
       </c>
       <c r="F57" t="n">
-        <v>-0.6175767503623835</v>
+        <v>-0.6175767503623837</v>
       </c>
       <c r="G57" t="n">
         <v>-0.07669649888473706</v>
@@ -2381,7 +2381,7 @@
         <v>-0.2709393764064</v>
       </c>
       <c r="J57" t="n">
-        <v>-0.06273060695693509</v>
+        <v>-0.06273060695693497</v>
       </c>
     </row>
     <row r="58">
@@ -2391,16 +2391,16 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>-0.3616693430372522</v>
+        <v>-0.3616693430372521</v>
       </c>
       <c r="C58" t="n">
         <v>0.3117449566605934</v>
       </c>
       <c r="D58" t="n">
-        <v>0.5105708082794717</v>
+        <v>0.5105708082794718</v>
       </c>
       <c r="E58" t="n">
-        <v>0.5538263737585842</v>
+        <v>0.5538263737585849</v>
       </c>
       <c r="F58" t="n">
         <v>0.2363746683536376</v>
@@ -2425,19 +2425,19 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>-0.3456799975872761</v>
+        <v>-0.3456799975872762</v>
       </c>
       <c r="C59" t="n">
         <v>1.153106105582694</v>
       </c>
       <c r="D59" t="n">
-        <v>0.3421817630241196</v>
+        <v>0.3421817630241197</v>
       </c>
       <c r="E59" t="n">
         <v>-0.002873768165734359</v>
       </c>
       <c r="F59" t="n">
-        <v>-0.05462703214188266</v>
+        <v>-0.05462703214188247</v>
       </c>
       <c r="G59" t="n">
         <v>13.0384048104053</v>
@@ -2449,7 +2449,7 @@
         <v>-0.2709393764064</v>
       </c>
       <c r="J59" t="n">
-        <v>0.9375317292849223</v>
+        <v>0.9375317292849228</v>
       </c>
     </row>
     <row r="60">
@@ -2496,10 +2496,10 @@
         <v>2.586446171029286</v>
       </c>
       <c r="C61" t="n">
-        <v>0.6148959543153059</v>
+        <v>0.6148959543153056</v>
       </c>
       <c r="D61" t="n">
-        <v>-0.1952578595486051</v>
+        <v>-0.1952578595486049</v>
       </c>
       <c r="E61" t="n">
         <v>2.252838028343252</v>
@@ -2530,10 +2530,10 @@
         <v>1.656385919567819</v>
       </c>
       <c r="C62" t="n">
-        <v>1.213582513560757</v>
+        <v>1.213582513560756</v>
       </c>
       <c r="D62" t="n">
-        <v>0.8765685523768122</v>
+        <v>0.8765685523768123</v>
       </c>
       <c r="E62" t="n">
         <v>1.512275190160361</v>
@@ -2561,13 +2561,13 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>0.4297847183650136</v>
+        <v>0.429784718365014</v>
       </c>
       <c r="C63" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D63" t="n">
-        <v>-0.1059150457714529</v>
+        <v>-0.1059150457714528</v>
       </c>
       <c r="E63" t="n">
         <v>0.4041337169669837</v>
@@ -2585,7 +2585,7 @@
         <v>-0.2709393764064</v>
       </c>
       <c r="J63" t="n">
-        <v>4.391406869852118</v>
+        <v>4.391406869852119</v>
       </c>
     </row>
     <row r="64">
@@ -2595,19 +2595,19 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>-0.3353869477172415</v>
+        <v>-0.3353869477172416</v>
       </c>
       <c r="C64" t="n">
         <v>0.9027481692136333</v>
       </c>
       <c r="D64" t="n">
-        <v>0.8473804479334588</v>
+        <v>0.8473804479334587</v>
       </c>
       <c r="E64" t="n">
         <v>0.2039274887477648</v>
       </c>
       <c r="F64" t="n">
-        <v>-0.2064149561657809</v>
+        <v>-0.2064149561657807</v>
       </c>
       <c r="G64" t="n">
         <v>-0.07669649888473706</v>
@@ -2632,10 +2632,10 @@
         <v>0.7883296848704492</v>
       </c>
       <c r="C65" t="n">
-        <v>0.451346025238293</v>
+        <v>0.4513460252382928</v>
       </c>
       <c r="D65" t="n">
-        <v>0.6269147842781521</v>
+        <v>0.6269147842781523</v>
       </c>
       <c r="E65" t="n">
         <v>0.6203564434437402</v>
@@ -2663,13 +2663,13 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>-0.3166876371501782</v>
+        <v>-0.316687637150178</v>
       </c>
       <c r="C66" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D66" t="n">
-        <v>0.3093106152329309</v>
+        <v>0.309310615232931</v>
       </c>
       <c r="E66" t="n">
         <v>-0.3157297504495348</v>
@@ -2684,7 +2684,7 @@
         <v>-0.1891480179719353</v>
       </c>
       <c r="I66" t="n">
-        <v>0.4761164870686064</v>
+        <v>0.4761164870686067</v>
       </c>
       <c r="J66" t="n">
         <v>-0.2883807434472616</v>
@@ -2697,13 +2697,13 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>-0.007388530268806459</v>
+        <v>-0.007388530268806158</v>
       </c>
       <c r="C67" t="n">
-        <v>0.9492778079101738</v>
+        <v>0.9492778079101736</v>
       </c>
       <c r="D67" t="n">
-        <v>-0.04688033142562327</v>
+        <v>-0.0468803314256231</v>
       </c>
       <c r="E67" t="n">
         <v>1.547025271201268</v>
@@ -2731,19 +2731,19 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>-0.3315895814270697</v>
+        <v>-0.3315895814270696</v>
       </c>
       <c r="C68" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D68" t="n">
-        <v>-0.082582020522232</v>
+        <v>-0.08258202052223183</v>
       </c>
       <c r="E68" t="n">
         <v>-0.5594675640707354</v>
       </c>
       <c r="F68" t="n">
-        <v>-0.184839749573755</v>
+        <v>-0.1848397495737549</v>
       </c>
       <c r="G68" t="n">
         <v>-0.07669649888473706</v>
@@ -2765,16 +2765,16 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>-0.4029026922142515</v>
+        <v>-0.4029026922142516</v>
       </c>
       <c r="C69" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D69" t="n">
-        <v>-1.059791339888413</v>
+        <v>-1.059791339888412</v>
       </c>
       <c r="E69" t="n">
-        <v>-0.560552293467776</v>
+        <v>-0.5605522934677759</v>
       </c>
       <c r="F69" t="n">
         <v>-0.1758777406816829</v>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>-0.3832198950406624</v>
+        <v>-0.3832198950406625</v>
       </c>
       <c r="C70" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D70" t="n">
-        <v>-0.7548436755287709</v>
+        <v>-0.7548436755287706</v>
       </c>
       <c r="E70" t="n">
         <v>-0.52156983076163</v>
@@ -2833,7 +2833,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>-0.3948428542033627</v>
+        <v>-0.3948428542033628</v>
       </c>
       <c r="C71" t="n">
         <v>-0.625979127747597</v>
@@ -2845,7 +2845,7 @@
         <v>-0.6229242337976095</v>
       </c>
       <c r="F71" t="n">
-        <v>-0.4261738461674132</v>
+        <v>-0.4261738461674131</v>
       </c>
       <c r="G71" t="n">
         <v>-0.07669649888473706</v>
@@ -2867,13 +2867,13 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>0.4726728722532237</v>
+        <v>0.472672872253224</v>
       </c>
       <c r="C72" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D72" t="n">
-        <v>-0.4695213559051455</v>
+        <v>-0.4695213559051453</v>
       </c>
       <c r="E72" t="n">
         <v>-0.5040017342353934</v>
@@ -2935,13 +2935,13 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>-0.4214082592290767</v>
+        <v>-0.4214082592290765</v>
       </c>
       <c r="C74" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D74" t="n">
-        <v>-0.9219726467954868</v>
+        <v>-0.9219726467954867</v>
       </c>
       <c r="E74" t="n">
         <v>-0.4427386284003125</v>
@@ -2969,13 +2969,13 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>-0.4146897616466616</v>
+        <v>-0.4146897616466615</v>
       </c>
       <c r="C75" t="n">
-        <v>0.1820147369918203</v>
+        <v>0.1820147369918201</v>
       </c>
       <c r="D75" t="n">
-        <v>-0.6518106156646839</v>
+        <v>-0.6518106156646837</v>
       </c>
       <c r="E75" t="n">
         <v>-0.5688685521784205</v>
@@ -3009,7 +3009,7 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D76" t="n">
-        <v>-0.5711614280134942</v>
+        <v>-0.571161428013494</v>
       </c>
       <c r="E76" t="n">
         <v>-0.6026533531904136</v>
@@ -3043,7 +3043,7 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D77" t="n">
-        <v>-0.2403577150645829</v>
+        <v>-0.2403577150645828</v>
       </c>
       <c r="E77" t="n">
         <v>-0.2039927012488939</v>
@@ -3061,7 +3061,7 @@
         <v>0.5359881890456704</v>
       </c>
       <c r="J77" t="n">
-        <v>0.9991206334174005</v>
+        <v>0.9991206334174008</v>
       </c>
     </row>
     <row r="78">
@@ -3071,13 +3071,13 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>-0.4519112825792901</v>
+        <v>-0.45191128257929</v>
       </c>
       <c r="C78" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D78" t="n">
-        <v>0.7262961881174264</v>
+        <v>0.7262961881174265</v>
       </c>
       <c r="E78" t="n">
         <v>-0.6278383866720814</v>
@@ -3105,13 +3105,13 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>-0.4202896620937888</v>
+        <v>-0.4202896620937889</v>
       </c>
       <c r="C79" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D79" t="n">
-        <v>-0.6153527637127763</v>
+        <v>-0.615352763712776</v>
       </c>
       <c r="E79" t="n">
         <v>-0.5553546317736231</v>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>-0.2244025889431489</v>
+        <v>-0.2244025889431487</v>
       </c>
       <c r="C80" t="n">
         <v>-0.625979127747597</v>
@@ -3173,13 +3173,13 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>-0.3150121023630614</v>
+        <v>-0.3150121023630613</v>
       </c>
       <c r="C81" t="n">
-        <v>0.3840132031766747</v>
+        <v>0.3840132031766745</v>
       </c>
       <c r="D81" t="n">
-        <v>0.06913519545637328</v>
+        <v>0.06913519545637346</v>
       </c>
       <c r="E81" t="n">
         <v>-0.1608353425367993</v>
@@ -3207,13 +3207,13 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>-0.3656222039166683</v>
+        <v>-0.3656222039166684</v>
       </c>
       <c r="C82" t="n">
         <v>1.056590462259494</v>
       </c>
       <c r="D82" t="n">
-        <v>0.8322334866627396</v>
+        <v>0.8322334866627398</v>
       </c>
       <c r="E82" t="n">
         <v>0.1068274680614436</v>
@@ -3228,7 +3228,7 @@
         <v>-0.1891480179719353</v>
       </c>
       <c r="I82" t="n">
-        <v>2.415147149774212</v>
+        <v>2.415147149774213</v>
       </c>
       <c r="J82" t="n">
         <v>0.8136852815276777</v>
@@ -3241,19 +3241,19 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>-0.3646310825530916</v>
+        <v>-0.3646310825530915</v>
       </c>
       <c r="C83" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D83" t="n">
-        <v>-0.3398934378539182</v>
+        <v>-0.339893437853918</v>
       </c>
       <c r="E83" t="n">
         <v>-0.4721373324388189</v>
       </c>
       <c r="F83" t="n">
-        <v>-0.4362476832303064</v>
+        <v>-0.4362476832303063</v>
       </c>
       <c r="G83" t="n">
         <v>-0.07669649888473706</v>
@@ -3278,10 +3278,10 @@
         <v>1.415259187707438</v>
       </c>
       <c r="C84" t="n">
-        <v>0.5860116693615292</v>
+        <v>0.5860116693615289</v>
       </c>
       <c r="D84" t="n">
-        <v>1.549209971332286</v>
+        <v>1.549209971332287</v>
       </c>
       <c r="E84" t="n">
         <v>0.4987311598005646</v>
@@ -3309,19 +3309,19 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>-0.39429738717138</v>
+        <v>-0.3942973871713801</v>
       </c>
       <c r="C85" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D85" t="n">
-        <v>-0.7125737022511967</v>
+        <v>-0.7125737022511965</v>
       </c>
       <c r="E85" t="n">
         <v>-0.532831431098961</v>
       </c>
       <c r="F85" t="n">
-        <v>-0.5537757822973934</v>
+        <v>-0.5537757822973935</v>
       </c>
       <c r="G85" t="n">
         <v>-0.07669649888473706</v>
@@ -3343,13 +3343,13 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>-0.4052476378384339</v>
+        <v>-0.405247637838434</v>
       </c>
       <c r="C86" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D86" t="n">
-        <v>-0.4283894203696599</v>
+        <v>-0.4283894203696597</v>
       </c>
       <c r="E86" t="n">
         <v>-0.4427386284003125</v>
@@ -3377,13 +3377,13 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>-0.369078628059377</v>
+        <v>-0.3690786280593769</v>
       </c>
       <c r="C87" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D87" t="n">
-        <v>-0.174999100921107</v>
+        <v>-0.1749991009211069</v>
       </c>
       <c r="E87" t="n">
         <v>-0.3706643862413937</v>
@@ -3411,19 +3411,19 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>-0.4320636139921374</v>
+        <v>-0.4320636139921375</v>
       </c>
       <c r="C88" t="n">
-        <v>0.9900086017312377</v>
+        <v>0.9900086017312379</v>
       </c>
       <c r="D88" t="n">
-        <v>-0.2008845520489836</v>
+        <v>-0.2008845520489835</v>
       </c>
       <c r="E88" t="n">
         <v>0.2161139548132824</v>
       </c>
       <c r="F88" t="n">
-        <v>0.04817248162012174</v>
+        <v>0.04817248162012193</v>
       </c>
       <c r="G88" t="n">
         <v>-0.07669649888473706</v>
@@ -3445,13 +3445,13 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>-0.4153603836456769</v>
+        <v>-0.4153603836456767</v>
       </c>
       <c r="C89" t="n">
-        <v>0.1820147369918203</v>
+        <v>0.1820147369918201</v>
       </c>
       <c r="D89" t="n">
-        <v>-0.09168543567628411</v>
+        <v>-0.09168543567628394</v>
       </c>
       <c r="E89" t="n">
         <v>-0.1484354729180606</v>
@@ -3485,10 +3485,10 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D90" t="n">
-        <v>-0.03810344114090468</v>
+        <v>-0.03810344114090451</v>
       </c>
       <c r="E90" t="n">
-        <v>-0.4948976194363722</v>
+        <v>-0.4948976194363723</v>
       </c>
       <c r="F90" t="n">
         <v>-1.000382558752324</v>
@@ -3519,7 +3519,7 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D91" t="n">
-        <v>-0.4727620538564262</v>
+        <v>-0.4727620538564261</v>
       </c>
       <c r="E91" t="n">
         <v>0.1338553088710381</v>
@@ -3531,7 +3531,7 @@
         <v>-0.07669649888473706</v>
       </c>
       <c r="H91" t="n">
-        <v>0.8842130728716947</v>
+        <v>0.884213072871695</v>
       </c>
       <c r="I91" t="n">
         <v>-0.2709393764064</v>
@@ -3547,13 +3547,13 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>-0.02240208149784883</v>
+        <v>-0.02240208149784895</v>
       </c>
       <c r="C92" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D92" t="n">
-        <v>-0.6477597432255832</v>
+        <v>-0.6477597432255829</v>
       </c>
       <c r="E92" t="n">
         <v>-0.2985901440824748</v>
@@ -3581,16 +3581,16 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>-0.1191836514040735</v>
+        <v>-0.1191836514040736</v>
       </c>
       <c r="C93" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D93" t="n">
-        <v>-0.5059792078570532</v>
+        <v>-0.505979207857053</v>
       </c>
       <c r="E93" t="n">
-        <v>-0.3886829467811234</v>
+        <v>-0.3886829467811233</v>
       </c>
       <c r="F93" t="n">
         <v>1.679258099977259</v>
@@ -3615,13 +3615,13 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>-0.4139780884747582</v>
+        <v>-0.4139780884747581</v>
       </c>
       <c r="C94" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D94" t="n">
-        <v>0.06519380605616706</v>
+        <v>0.06519380605616724</v>
       </c>
       <c r="E94" t="n">
         <v>-0.4067015073208531</v>
@@ -3649,13 +3649,13 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>-0.3802075541452409</v>
+        <v>-0.3802075541452407</v>
       </c>
       <c r="C95" t="n">
-        <v>0.1820147369918203</v>
+        <v>0.1820147369918201</v>
       </c>
       <c r="D95" t="n">
-        <v>0.8429613143635308</v>
+        <v>0.8429613143635311</v>
       </c>
       <c r="E95" t="n">
         <v>-0.574874739024997</v>
@@ -3683,13 +3683,13 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>-0.3518038771201261</v>
+        <v>-0.3518038771201258</v>
       </c>
       <c r="C96" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D96" t="n">
-        <v>-0.4509609949114472</v>
+        <v>-0.450960994911447</v>
       </c>
       <c r="E96" t="n">
         <v>0.512245080205362</v>
@@ -3717,10 +3717,10 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>0.0287804795102509</v>
+        <v>0.02878047951025078</v>
       </c>
       <c r="C97" t="n">
-        <v>0.06998890547318484</v>
+        <v>0.06998890547318509</v>
       </c>
       <c r="D97" t="n">
         <v>3.624325556027908</v>
@@ -3757,7 +3757,7 @@
         <v>0.6243196514633232</v>
       </c>
       <c r="D98" t="n">
-        <v>-0.3919151681244765</v>
+        <v>-0.3919151681244764</v>
       </c>
       <c r="E98" t="n">
         <v>0.3500780353477946</v>
@@ -3819,13 +3819,13 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>-0.04026944824976752</v>
+        <v>-0.04026944824976722</v>
       </c>
       <c r="C100" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D100" t="n">
-        <v>-0.2489046107602682</v>
+        <v>-0.248904610760268</v>
       </c>
       <c r="E100" t="n">
         <v>-0.2084973413838263</v>
@@ -3853,13 +3853,13 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>0.2900011056923293</v>
+        <v>0.2900011056923297</v>
       </c>
       <c r="C101" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D101" t="n">
-        <v>-0.7236846666555876</v>
+        <v>-0.7236846666555874</v>
       </c>
       <c r="E101" t="n">
         <v>0.8365791699204966</v>
@@ -3887,13 +3887,13 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>-0.3489338631191425</v>
+        <v>-0.3489338631191427</v>
       </c>
       <c r="C102" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D102" t="n">
-        <v>-0.9953982507266018</v>
+        <v>-0.9953982507266015</v>
       </c>
       <c r="E102" t="n">
         <v>-0.4787757494797719</v>
@@ -3921,13 +3921,13 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>-0.2949169609493779</v>
+        <v>-0.2949169609493776</v>
       </c>
       <c r="C103" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D103" t="n">
-        <v>-0.5952380867737926</v>
+        <v>-0.5952380867737925</v>
       </c>
       <c r="E103" t="n">
         <v>0.3680965958875242</v>
@@ -3955,16 +3955,16 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>0.1614001820334599</v>
+        <v>0.1614001820334603</v>
       </c>
       <c r="C104" t="n">
-        <v>0.06998890547318484</v>
+        <v>0.06998890547318509</v>
       </c>
       <c r="D104" t="n">
-        <v>-0.03569584714408063</v>
+        <v>-0.03569584714408046</v>
       </c>
       <c r="E104" t="n">
-        <v>0.9601350136215003</v>
+        <v>0.9601350136215</v>
       </c>
       <c r="F104" t="n">
         <v>1.679258099977259</v>
@@ -3995,7 +3995,7 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D105" t="n">
-        <v>-0.8097946407896172</v>
+        <v>-0.809794640789617</v>
       </c>
       <c r="E105" t="n">
         <v>-0.4607571889400422</v>
@@ -4023,13 +4023,13 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>0.1644142661817149</v>
+        <v>0.1644142661817148</v>
       </c>
       <c r="C106" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D106" t="n">
-        <v>-0.2499361326545751</v>
+        <v>-0.249936132654575</v>
       </c>
       <c r="E106" t="n">
         <v>1.831203711713576</v>
@@ -4063,7 +4063,7 @@
         <v>1.110098128925304</v>
       </c>
       <c r="D107" t="n">
-        <v>-0.1479689519646148</v>
+        <v>-0.1479689519646147</v>
       </c>
       <c r="E107" t="n">
         <v>9.204398684570972</v>
@@ -4091,13 +4091,13 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>0.4389899806629712</v>
+        <v>0.4389899806629711</v>
       </c>
       <c r="C108" t="n">
         <v>1.413170352121563</v>
       </c>
       <c r="D108" t="n">
-        <v>-0.06443411199506029</v>
+        <v>-0.06443411199506011</v>
       </c>
       <c r="E108" t="n">
         <v>0.04376250617238961</v>
@@ -4131,7 +4131,7 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D109" t="n">
-        <v>-0.2526438776271307</v>
+        <v>-0.2526438776271305</v>
       </c>
       <c r="E109" t="n">
         <v>-0.1985296270426992</v>
@@ -4165,7 +4165,7 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D110" t="n">
-        <v>-0.06958976782664315</v>
+        <v>-0.06958976782664299</v>
       </c>
       <c r="E110" t="n">
         <v>-0.1173446233593113</v>
@@ -4199,7 +4199,7 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D111" t="n">
-        <v>-0.1681364464360421</v>
+        <v>-0.1681364464360419</v>
       </c>
       <c r="E111" t="n">
         <v>-0.1364230992249075</v>
@@ -4233,7 +4233,7 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D112" t="n">
-        <v>-0.0320271324822534</v>
+        <v>-0.03202713248225323</v>
       </c>
       <c r="E112" t="n">
         <v>-0.352645825701664</v>
@@ -4264,10 +4264,10 @@
         <v>3.826526506311243</v>
       </c>
       <c r="C113" t="n">
-        <v>0.9900086017312377</v>
+        <v>0.9900086017312379</v>
       </c>
       <c r="D113" t="n">
-        <v>-0.2566410249675696</v>
+        <v>-0.2566410249675695</v>
       </c>
       <c r="E113" t="n">
         <v>-0.1544416597646372</v>
@@ -4295,13 +4295,13 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>-0.3489338631191425</v>
+        <v>-0.3489338631191427</v>
       </c>
       <c r="C114" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D114" t="n">
-        <v>-1.101457456404879</v>
+        <v>-1.101457456404878</v>
       </c>
       <c r="E114" t="n">
         <v>-0.6529551680304924</v>
@@ -4329,13 +4329,13 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>-0.07972654982692028</v>
+        <v>-0.0797265498269204</v>
       </c>
       <c r="C115" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D115" t="n">
-        <v>0.4151891847944807</v>
+        <v>0.4151891847944809</v>
       </c>
       <c r="E115" t="n">
         <v>-0.5868871127181502</v>
@@ -4363,13 +4363,13 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>-0.3217068276407891</v>
+        <v>-0.321706827640789</v>
       </c>
       <c r="C116" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D116" t="n">
-        <v>-0.06443411199506029</v>
+        <v>-0.06443411199506011</v>
       </c>
       <c r="E116" t="n">
         <v>-0.5472462795307448</v>
@@ -4397,13 +4397,13 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>-0.2424870938326771</v>
+        <v>-0.2424870938326772</v>
       </c>
       <c r="C117" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D117" t="n">
-        <v>-0.7773876612768102</v>
+        <v>-0.7773876612768101</v>
       </c>
       <c r="E117" t="n">
         <v>-0.5796796885022582</v>
@@ -4431,13 +4431,13 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>-0.4309248737884517</v>
+        <v>-0.4309248737884516</v>
       </c>
       <c r="C118" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D118" t="n">
-        <v>-0.4695213559051455</v>
+        <v>-0.4695213559051453</v>
       </c>
       <c r="E118" t="n">
         <v>-0.5040017342353934</v>
@@ -4465,13 +4465,13 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>-0.1946163455956902</v>
+        <v>-0.1946163455956899</v>
       </c>
       <c r="C119" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D119" t="n">
-        <v>-0.7125737022511967</v>
+        <v>-0.7125737022511965</v>
       </c>
       <c r="E119" t="n">
         <v>-0.655357642769123</v>
@@ -4499,13 +4499,13 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>-0.4453268108368488</v>
+        <v>-0.4453268108368487</v>
       </c>
       <c r="C120" t="n">
-        <v>1.25933988997771</v>
+        <v>1.259339889977711</v>
       </c>
       <c r="D120" t="n">
-        <v>0.3151905051549626</v>
+        <v>0.3151905051549627</v>
       </c>
       <c r="E120" t="n">
         <v>-0.5688685521784205</v>
@@ -4536,10 +4536,10 @@
         <v>-0.3214637291097322</v>
       </c>
       <c r="C121" t="n">
-        <v>0.1820147369918203</v>
+        <v>0.1820147369918201</v>
       </c>
       <c r="D121" t="n">
-        <v>0.7092825238732027</v>
+        <v>0.7092825238732029</v>
       </c>
       <c r="E121" t="n">
         <v>-0.1827565406127839</v>
@@ -4567,13 +4567,13 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>-0.4107490729828216</v>
+        <v>-0.4107490729828214</v>
       </c>
       <c r="C122" t="n">
-        <v>0.5418339031364962</v>
+        <v>0.5418339031364959</v>
       </c>
       <c r="D122" t="n">
-        <v>0.08371208006348518</v>
+        <v>0.08371208006348536</v>
       </c>
       <c r="E122" t="n">
         <v>-0.4705854946889856</v>
@@ -4607,7 +4607,7 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D123" t="n">
-        <v>-0.2403577150645829</v>
+        <v>-0.2403577150645828</v>
       </c>
       <c r="E123" t="n">
         <v>-0.3742680983493396</v>
@@ -4635,13 +4635,13 @@
         </is>
       </c>
       <c r="B124" t="n">
-        <v>-0.4236210325824282</v>
+        <v>-0.4236210325824278</v>
       </c>
       <c r="C124" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D124" t="n">
-        <v>0.7019909534828213</v>
+        <v>0.7019909534828214</v>
       </c>
       <c r="E124" t="n">
         <v>-0.3443295669910195</v>
@@ -4669,19 +4669,19 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>-0.428928325022768</v>
+        <v>-0.4289283250227678</v>
       </c>
       <c r="C125" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D125" t="n">
-        <v>-0.4070221811304465</v>
+        <v>-0.4070221811304464</v>
       </c>
       <c r="E125" t="n">
         <v>-0.5508499916386906</v>
       </c>
       <c r="F125" t="n">
-        <v>-0.5537757822973934</v>
+        <v>-0.5537757822973935</v>
       </c>
       <c r="G125" t="n">
         <v>-0.07669649888473706</v>
@@ -4703,13 +4703,13 @@
         </is>
       </c>
       <c r="B126" t="n">
-        <v>-0.1118767807416381</v>
+        <v>-0.1118767807416378</v>
       </c>
       <c r="C126" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D126" t="n">
-        <v>-0.5991492739563729</v>
+        <v>-0.5991492739563727</v>
       </c>
       <c r="E126" t="n">
         <v>-0.4175126436446909</v>
@@ -4743,7 +4743,7 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D127" t="n">
-        <v>-0.9556260485972479</v>
+        <v>-0.9556260485972478</v>
       </c>
       <c r="E127" t="n">
         <v>-0.5688685521784205</v>
@@ -4771,13 +4771,13 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>-0.1898530870646467</v>
+        <v>-0.1898530870646465</v>
       </c>
       <c r="C128" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D128" t="n">
-        <v>-0.3236899480975148</v>
+        <v>-0.3236899480975147</v>
       </c>
       <c r="E128" t="n">
         <v>-0.5472462795307448</v>
@@ -4805,19 +4805,19 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>-0.2982797153003719</v>
+        <v>-0.2982797153003716</v>
       </c>
       <c r="C129" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D129" t="n">
-        <v>-0.4816739732224481</v>
+        <v>-0.4816739732224479</v>
       </c>
       <c r="E129" t="n">
-        <v>-0.4298682280147913</v>
+        <v>-0.4298682280147912</v>
       </c>
       <c r="F129" t="n">
-        <v>-0.6175767503623835</v>
+        <v>-0.6175767503623837</v>
       </c>
       <c r="G129" t="n">
         <v>-0.07669649888473706</v>
@@ -4839,19 +4839,19 @@
         </is>
       </c>
       <c r="B130" t="n">
-        <v>-0.4339700867806267</v>
+        <v>-0.4339700867806264</v>
       </c>
       <c r="C130" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D130" t="n">
-        <v>-0.7275307697186459</v>
+        <v>-0.7275307697186458</v>
       </c>
       <c r="E130" t="n">
         <v>-0.5832834006102042</v>
       </c>
       <c r="F130" t="n">
-        <v>-0.6430971375883794</v>
+        <v>-0.6430971375883796</v>
       </c>
       <c r="G130" t="n">
         <v>-0.07669649888473706</v>
@@ -4879,13 +4879,13 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D131" t="n">
-        <v>-1.101457456404879</v>
+        <v>-1.101457456404878</v>
       </c>
       <c r="E131" t="n">
         <v>-0.6679706351469339</v>
       </c>
       <c r="F131" t="n">
-        <v>-0.5537757822973934</v>
+        <v>-0.5537757822973935</v>
       </c>
       <c r="G131" t="n">
         <v>-0.07669649888473706</v>
@@ -4907,13 +4907,13 @@
         </is>
       </c>
       <c r="B132" t="n">
-        <v>-0.2785670173807512</v>
+        <v>-0.2785670173807514</v>
       </c>
       <c r="C132" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D132" t="n">
-        <v>-0.3685611504998627</v>
+        <v>-0.3685611504998625</v>
       </c>
       <c r="E132" t="n">
         <v>-0.5492119406805334</v>
@@ -4941,13 +4941,13 @@
         </is>
       </c>
       <c r="B133" t="n">
-        <v>-0.3281505380462335</v>
+        <v>-0.3281505380462334</v>
       </c>
       <c r="C133" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D133" t="n">
-        <v>-0.06941980115087652</v>
+        <v>-0.0694198011508767</v>
       </c>
       <c r="E133" t="n">
         <v>-0.5688685521784205</v>
@@ -4975,13 +4975,13 @@
         </is>
       </c>
       <c r="B134" t="n">
-        <v>-0.4165261462641617</v>
+        <v>-0.4165261462641615</v>
       </c>
       <c r="C134" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D134" t="n">
-        <v>-0.5375760128820398</v>
+        <v>-0.5375760128820397</v>
       </c>
       <c r="E134" t="n">
         <v>-0.5904908248260961</v>
@@ -5009,13 +5009,13 @@
         </is>
       </c>
       <c r="B135" t="n">
-        <v>-0.4000355097916702</v>
+        <v>-0.4000355097916704</v>
       </c>
       <c r="C135" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D135" t="n">
-        <v>-0.6523893117274127</v>
+        <v>-0.6523893117274125</v>
       </c>
       <c r="E135" t="n">
         <v>0.079799627251849</v>
@@ -5043,13 +5043,13 @@
         </is>
       </c>
       <c r="B136" t="n">
-        <v>-0.130788681279707</v>
+        <v>-0.1307886812797069</v>
       </c>
       <c r="C136" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D136" t="n">
-        <v>-0.05363178549079121</v>
+        <v>-0.05363178549079103</v>
       </c>
       <c r="E136" t="n">
         <v>-0.5148128705592313</v>
@@ -5080,16 +5080,16 @@
         <v>-0.2985341131184062</v>
       </c>
       <c r="C137" t="n">
-        <v>0.765956938693967</v>
+        <v>0.7659569386939667</v>
       </c>
       <c r="D137" t="n">
-        <v>-0.9502248853451134</v>
+        <v>-0.9502248853451133</v>
       </c>
       <c r="E137" t="n">
         <v>-0.595896392988015</v>
       </c>
       <c r="F137" t="n">
-        <v>-0.5537757822973934</v>
+        <v>-0.5537757822973935</v>
       </c>
       <c r="G137" t="n">
         <v>-0.07669649888473706</v>
@@ -5111,19 +5111,19 @@
         </is>
       </c>
       <c r="B138" t="n">
-        <v>-0.0868417648654234</v>
+        <v>-0.08684176486542346</v>
       </c>
       <c r="C138" t="n">
         <v>-0.3381659059882294</v>
       </c>
       <c r="D138" t="n">
-        <v>-0.8023161070558925</v>
+        <v>-0.8023161070558922</v>
       </c>
       <c r="E138" t="n">
         <v>-0.4427386284003125</v>
       </c>
       <c r="F138" t="n">
-        <v>-0.5537757822973934</v>
+        <v>-0.5537757822973935</v>
       </c>
       <c r="G138" t="n">
         <v>-0.07669649888473706</v>
@@ -5145,13 +5145,13 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>-0.4052476378384339</v>
+        <v>-0.405247637838434</v>
       </c>
       <c r="C139" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D139" t="n">
-        <v>0.1624147445945875</v>
+        <v>0.1624147445945877</v>
       </c>
       <c r="E139" t="n">
         <v>-0.6409427943373392</v>
@@ -5179,13 +5179,13 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>-0.3649450269417707</v>
+        <v>-0.3649450269417704</v>
       </c>
       <c r="C140" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D140" t="n">
-        <v>-1.101457456404879</v>
+        <v>-1.101457456404878</v>
       </c>
       <c r="E140" t="n">
         <v>-0.6769799154167987</v>
@@ -5213,19 +5213,19 @@
         </is>
       </c>
       <c r="B141" t="n">
-        <v>-0.4219410269672297</v>
+        <v>-0.4219410269672296</v>
       </c>
       <c r="C141" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D141" t="n">
-        <v>-0.7773876612768102</v>
+        <v>-0.7773876612768101</v>
       </c>
       <c r="E141" t="n">
         <v>-0.6180100809231378</v>
       </c>
       <c r="F141" t="n">
-        <v>-0.513175166256036</v>
+        <v>-0.5131751662560361</v>
       </c>
       <c r="G141" t="n">
         <v>-0.07669649888473706</v>
@@ -5247,13 +5247,13 @@
         </is>
       </c>
       <c r="B142" t="n">
-        <v>-0.4269490437058681</v>
+        <v>-0.4269490437058683</v>
       </c>
       <c r="C142" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D142" t="n">
-        <v>-0.1292480710206739</v>
+        <v>-0.1292480710206737</v>
       </c>
       <c r="E142" t="n">
         <v>-0.669257675185486</v>
@@ -5287,7 +5287,7 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D143" t="n">
-        <v>-0.4602129681727435</v>
+        <v>-0.4602129681727434</v>
       </c>
       <c r="E143" t="n">
         <v>-0.1688565081964209</v>
@@ -5315,13 +5315,13 @@
         </is>
       </c>
       <c r="B144" t="n">
-        <v>-0.2400432418205789</v>
+        <v>-0.2400432418205788</v>
       </c>
       <c r="C144" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D144" t="n">
-        <v>-0.3613238597898066</v>
+        <v>-0.3613238597898064</v>
       </c>
       <c r="E144" t="n">
         <v>0.28057787326598</v>
@@ -5352,16 +5352,16 @@
         <v>-0.3273622241424277</v>
       </c>
       <c r="C145" t="n">
-        <v>0.4179729220835761</v>
+        <v>0.4179729220835757</v>
       </c>
       <c r="D145" t="n">
-        <v>0.1732170710988565</v>
+        <v>0.1732170710988566</v>
       </c>
       <c r="E145" t="n">
         <v>-0.2599789429259112</v>
       </c>
       <c r="F145" t="n">
-        <v>-0.4261738461674132</v>
+        <v>-0.4261738461674131</v>
       </c>
       <c r="G145" t="n">
         <v>-0.07669649888473706</v>
@@ -5383,13 +5383,13 @@
         </is>
       </c>
       <c r="B146" t="n">
-        <v>-0.3673034619352516</v>
+        <v>-0.3673034619352515</v>
       </c>
       <c r="C146" t="n">
-        <v>1.394005534100946</v>
+        <v>1.394005534100947</v>
       </c>
       <c r="D146" t="n">
-        <v>-0.6698913389904267</v>
+        <v>-0.6698913389904266</v>
       </c>
       <c r="E146" t="n">
         <v>-0.2740193797101161</v>
@@ -5423,10 +5423,10 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D147" t="n">
-        <v>-0.6503523015866076</v>
+        <v>-0.6503523015866075</v>
       </c>
       <c r="E147" t="n">
-        <v>-0.3766705730879703</v>
+        <v>-0.3766705730879702</v>
       </c>
       <c r="F147" t="n">
         <v>-1.000382558752324</v>
@@ -5451,13 +5451,13 @@
         </is>
       </c>
       <c r="B148" t="n">
-        <v>-0.2400432418205789</v>
+        <v>-0.2400432418205788</v>
       </c>
       <c r="C148" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D148" t="n">
-        <v>-0.3524961521088986</v>
+        <v>-0.3524961521088985</v>
       </c>
       <c r="E148" t="n">
         <v>-0.2599789429259112</v>
@@ -5485,13 +5485,13 @@
         </is>
       </c>
       <c r="B149" t="n">
-        <v>-0.3258637072844</v>
+        <v>-0.3258637072843997</v>
       </c>
       <c r="C149" t="n">
-        <v>0.3082712969596775</v>
+        <v>0.3082712969596774</v>
       </c>
       <c r="D149" t="n">
-        <v>-0.571603341370487</v>
+        <v>-0.5716033413704869</v>
       </c>
       <c r="E149" t="n">
         <v>0.1879109904902272</v>
@@ -5519,13 +5519,13 @@
         </is>
       </c>
       <c r="B150" t="n">
-        <v>-0.2853188159394553</v>
+        <v>-0.2853188159394554</v>
       </c>
       <c r="C150" t="n">
-        <v>0.9900086017312377</v>
+        <v>0.9900086017312379</v>
       </c>
       <c r="D150" t="n">
-        <v>0.1242647560541947</v>
+        <v>0.1242647560541948</v>
       </c>
       <c r="E150" t="n">
         <v>-0.01999547727588479</v>
@@ -5553,13 +5553,13 @@
         </is>
       </c>
       <c r="B151" t="n">
-        <v>-0.3405763659890975</v>
+        <v>-0.3405763659890976</v>
       </c>
       <c r="C151" t="n">
         <v>1.874686103819593</v>
       </c>
       <c r="D151" t="n">
-        <v>0.3151905051549626</v>
+        <v>0.3151905051549627</v>
       </c>
       <c r="E151" t="n">
         <v>0.17439707008543</v>
@@ -5587,16 +5587,16 @@
         </is>
       </c>
       <c r="B152" t="n">
-        <v>-0.3015631431384707</v>
+        <v>-0.3015631431384704</v>
       </c>
       <c r="C152" t="n">
-        <v>1.071774575346107</v>
+        <v>1.071774575346108</v>
       </c>
       <c r="D152" t="n">
-        <v>-0.1292480710206739</v>
+        <v>-0.1292480710206737</v>
       </c>
       <c r="E152" t="n">
-        <v>0.3746487997201534</v>
+        <v>0.3746487997201532</v>
       </c>
       <c r="F152" t="n">
         <v>0.2176359224883957</v>
@@ -5621,13 +5621,13 @@
         </is>
       </c>
       <c r="B153" t="n">
-        <v>-0.3682703820307945</v>
+        <v>-0.3682703820307947</v>
       </c>
       <c r="C153" t="n">
         <v>0.9033829821542733</v>
       </c>
       <c r="D153" t="n">
-        <v>-0.1204098038808174</v>
+        <v>-0.1204098038808172</v>
       </c>
       <c r="E153" t="n">
         <v>0.1158367483313084</v>
@@ -5655,13 +5655,13 @@
         </is>
       </c>
       <c r="B154" t="n">
-        <v>-0.2865148151605872</v>
+        <v>-0.286514815160587</v>
       </c>
       <c r="C154" t="n">
         <v>1.402478570538486</v>
       </c>
       <c r="D154" t="n">
-        <v>0.3737082510180881</v>
+        <v>0.3737082510180882</v>
       </c>
       <c r="E154" t="n">
         <v>0.1338553088710381</v>
@@ -5695,10 +5695,10 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D155" t="n">
-        <v>-0.06443411199506029</v>
+        <v>-0.06443411199506011</v>
       </c>
       <c r="E155" t="n">
-        <v>-0.4289597291640486</v>
+        <v>-0.4289597291640487</v>
       </c>
       <c r="F155" t="n">
         <v>-1.000382558752324</v>
@@ -5723,16 +5723,16 @@
         </is>
       </c>
       <c r="B156" t="n">
-        <v>-0.4065093474818898</v>
+        <v>-0.4065093474818895</v>
       </c>
       <c r="C156" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D156" t="n">
-        <v>1.940724597517353</v>
+        <v>1.940724597517354</v>
       </c>
       <c r="E156" t="n">
-        <v>0.4359311767429774</v>
+        <v>0.435931176742977</v>
       </c>
       <c r="F156" t="n">
         <v>-1.000382558752324</v>
@@ -5757,13 +5757,13 @@
         </is>
       </c>
       <c r="B157" t="n">
-        <v>-0.01295299331173842</v>
+        <v>-0.01295299331173805</v>
       </c>
       <c r="C157" t="n">
-        <v>0.5860116693615292</v>
+        <v>0.5860116693615289</v>
       </c>
       <c r="D157" t="n">
-        <v>-0.2657710910959026</v>
+        <v>-0.2657710910959024</v>
       </c>
       <c r="E157" t="n">
         <v>0.1698924299504975</v>
@@ -5791,13 +5791,13 @@
         </is>
       </c>
       <c r="B158" t="n">
-        <v>-0.3636917542624964</v>
+        <v>-0.3636917542624962</v>
       </c>
       <c r="C158" t="n">
         <v>0.3117449566605934</v>
       </c>
       <c r="D158" t="n">
-        <v>0.8749580789457956</v>
+        <v>0.8749580789457968</v>
       </c>
       <c r="E158" t="n">
         <v>-0.01999547727588479</v>
@@ -5831,7 +5831,7 @@
         <v>-0.116191757780307</v>
       </c>
       <c r="D159" t="n">
-        <v>-0.06652488486685428</v>
+        <v>-0.06652488486685409</v>
       </c>
       <c r="E159" t="n">
         <v>-0.1184045386851777</v>
@@ -5859,19 +5859,19 @@
         </is>
       </c>
       <c r="B160" t="n">
-        <v>-0.4187485124564233</v>
+        <v>-0.4187485124564231</v>
       </c>
       <c r="C160" t="n">
-        <v>0.5860116693615292</v>
+        <v>0.5860116693615289</v>
       </c>
       <c r="D160" t="n">
-        <v>0.4088585190291882</v>
+        <v>0.4088585190291883</v>
       </c>
       <c r="E160" t="n">
         <v>-0.1876337449694024</v>
       </c>
       <c r="F160" t="n">
-        <v>-0.7183151209913151</v>
+        <v>-0.7183151209913153</v>
       </c>
       <c r="G160" t="n">
         <v>-0.07669649888473706</v>
@@ -5893,13 +5893,13 @@
         </is>
       </c>
       <c r="B161" t="n">
-        <v>-0.1042941791108083</v>
+        <v>-0.1042941791108082</v>
       </c>
       <c r="C161" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D161" t="n">
-        <v>0.1192054385775118</v>
+        <v>0.1192054385775119</v>
       </c>
       <c r="E161" t="n">
         <v>-0.287779007758637</v>
@@ -5927,13 +5927,13 @@
         </is>
       </c>
       <c r="B162" t="n">
-        <v>-0.0712988193929654</v>
+        <v>-0.07129881939296551</v>
       </c>
       <c r="C162" t="n">
-        <v>0.9900086017312377</v>
+        <v>0.9900086017312379</v>
       </c>
       <c r="D162" t="n">
-        <v>-0.545909236185333</v>
+        <v>-0.5459092361853328</v>
       </c>
       <c r="E162" t="n">
         <v>-0.6409427943373392</v>
@@ -5967,7 +5967,7 @@
         <v>-0.625979127747597</v>
       </c>
       <c r="D163" t="n">
-        <v>-1.101457456404879</v>
+        <v>-1.101457456404878</v>
       </c>
       <c r="E163" t="n">
         <v>-0.6649675417236456</v>
@@ -5995,13 +5995,13 @@
         </is>
       </c>
       <c r="B164" t="n">
-        <v>0.1539808979762175</v>
+        <v>0.1539808979762178</v>
       </c>
       <c r="C164" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D164" t="n">
-        <v>-1.101457456404879</v>
+        <v>-1.101457456404878</v>
       </c>
       <c r="E164" t="n">
         <v>-0.658961354877069</v>
@@ -6029,13 +6029,13 @@
         </is>
       </c>
       <c r="B165" t="n">
-        <v>-0.402853173776406</v>
+        <v>-0.4028531737764059</v>
       </c>
       <c r="C165" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D165" t="n">
-        <v>-0.4332844606317342</v>
+        <v>-0.433284460631734</v>
       </c>
       <c r="E165" t="n">
         <v>-0.4067015073208531</v>
@@ -6063,13 +6063,13 @@
         </is>
       </c>
       <c r="B166" t="n">
-        <v>-0.3130909827849463</v>
+        <v>-0.3130909827849462</v>
       </c>
       <c r="C166" t="n">
-        <v>2.605996331210072</v>
+        <v>2.605996331210073</v>
       </c>
       <c r="D166" t="n">
-        <v>-0.4070221811304465</v>
+        <v>-0.4070221811304464</v>
       </c>
       <c r="E166" t="n">
         <v>-0.4247200678605828</v>
@@ -6097,19 +6097,19 @@
         </is>
       </c>
       <c r="B167" t="n">
-        <v>-0.365368986030756</v>
+        <v>-0.3653689860307557</v>
       </c>
       <c r="C167" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D167" t="n">
-        <v>-0.7203513773342703</v>
+        <v>-0.7203513773342701</v>
       </c>
       <c r="E167" t="n">
         <v>-0.4517479086701774</v>
       </c>
       <c r="F167" t="n">
-        <v>-0.5537757822973934</v>
+        <v>-0.5537757822973935</v>
       </c>
       <c r="G167" t="n">
         <v>-0.07669649888473706</v>
@@ -6131,16 +6131,16 @@
         </is>
       </c>
       <c r="B168" t="n">
-        <v>-0.3519459392166659</v>
+        <v>-0.3519459392166658</v>
       </c>
       <c r="C168" t="n">
         <v>0.7838363106335547</v>
       </c>
       <c r="D168" t="n">
-        <v>-0.08960458151957031</v>
+        <v>-0.08960458151957014</v>
       </c>
       <c r="E168" t="n">
-        <v>-0.02195224403133055</v>
+        <v>-0.02195224403133064</v>
       </c>
       <c r="F168" t="n">
         <v>-0.6851307165488435</v>
@@ -6168,7 +6168,7 @@
         <v>-0.4064989544864739</v>
       </c>
       <c r="C169" t="n">
-        <v>0.2755576270462177</v>
+        <v>0.2755576270462178</v>
       </c>
       <c r="D169" t="n">
         <v>4.556053313157821</v>
@@ -6199,13 +6199,13 @@
         </is>
       </c>
       <c r="B170" t="n">
-        <v>-0.3860993385436392</v>
+        <v>-0.3860993385436391</v>
       </c>
       <c r="C170" t="n">
-        <v>0.9368943462660535</v>
+        <v>0.9368943462660532</v>
       </c>
       <c r="D170" t="n">
-        <v>0.3609074941105293</v>
+        <v>0.3609074941105295</v>
       </c>
       <c r="E170" t="n">
         <v>-0.2052212394675118</v>
@@ -6233,13 +6233,13 @@
         </is>
       </c>
       <c r="B171" t="n">
-        <v>-0.3992857131495787</v>
+        <v>-0.3992857131495784</v>
       </c>
       <c r="C171" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D171" t="n">
-        <v>-0.8514607573060831</v>
+        <v>-0.8514607573060829</v>
       </c>
       <c r="E171" t="n">
         <v>-0.6139149535277447</v>
@@ -6257,7 +6257,7 @@
         <v>-0.2709393764064</v>
       </c>
       <c r="J171" t="n">
-        <v>-0.0518200509068534</v>
+        <v>-0.05182005090685327</v>
       </c>
     </row>
     <row r="172">
@@ -6267,13 +6267,13 @@
         </is>
       </c>
       <c r="B172" t="n">
-        <v>-0.4089169576710922</v>
+        <v>-0.4089169576710919</v>
       </c>
       <c r="C172" t="n">
         <v>-0.625979127747597</v>
       </c>
       <c r="D172" t="n">
-        <v>-0.9070155793280377</v>
+        <v>-0.9070155793280374</v>
       </c>
       <c r="E172" t="n">
         <v>-0.5580574158545826</v>

</xml_diff>